<commit_message>
Utilizes FortniteStats and bug fixes
</commit_message>
<xml_diff>
--- a/generated/fortnite_stats.xlsx
+++ b/generated/fortnite_stats.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,18 +442,42 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2.48</v>
+        <v>4.57</v>
       </c>
       <c r="B2" t="n">
-        <v>612.2833333333333</v>
+        <v>350.09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="B3" t="n">
+        <v>381.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="B4" t="n">
+        <v>325.11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="B5" t="n">
+        <v>112.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>2.48</v>
       </c>
-      <c r="B3" t="n">
-        <v>612.28</v>
+      <c r="B6" t="n">
+        <v>612.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>